<commit_message>
Portfolio za regularne i iregularne
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\ferprogrami\.vscode\PROJEKT R\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\FER\5.sem\SAP\github projekt\Projekt-R\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7AA356E-5862-4606-8260-83253054EB56}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E97FDC70-5356-4619-83F7-4E4BC8E27430}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3240" yWindow="3240" windowWidth="21600" windowHeight="11235" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="List1" sheetId="1" r:id="rId1"/>
@@ -207,99 +207,57 @@
     <t>ULPL</t>
   </si>
   <si>
-    <t>18.3.2019</t>
-  </si>
-  <si>
     <t>INGR;VLEN;KRAS</t>
   </si>
   <si>
-    <t>22.10.2018</t>
-  </si>
-  <si>
     <t>ULPL;IGH;JDPL;LKRI</t>
   </si>
   <si>
-    <t>24.9.2018</t>
-  </si>
-  <si>
     <t>LKPC</t>
   </si>
   <si>
     <t>MAIS;LKRI;VLEN;JDPL</t>
   </si>
   <si>
-    <t>19.3.2018</t>
-  </si>
-  <si>
     <t>MAIS;PTKM;ZB</t>
   </si>
   <si>
     <t>IGH</t>
   </si>
   <si>
-    <t>18.9.2017</t>
-  </si>
-  <si>
     <t>VDKT-R-A</t>
   </si>
   <si>
-    <t>19.6.2017</t>
-  </si>
-  <si>
     <t>LEDO-R-A;BLJE-R-A;VPIK-R-A</t>
   </si>
   <si>
-    <t>22.5.2017</t>
-  </si>
-  <si>
     <t>HIMR-R-A;LKRI;VART;TPNG</t>
   </si>
   <si>
-    <t>20.3.2017</t>
-  </si>
-  <si>
     <t>SUNH-R-A</t>
   </si>
   <si>
-    <t>21.11.2016</t>
-  </si>
-  <si>
     <t>MAIS;INA</t>
   </si>
   <si>
     <t>HIMR-R-A;LKPC-R-A;	SUNH-R-A;ULPL-R-A</t>
   </si>
   <si>
-    <t>19.9.2016</t>
-  </si>
-  <si>
     <t>RIZO;LKPC;PTKM</t>
   </si>
   <si>
     <t>LEDO-R-A;VART-R-A</t>
   </si>
   <si>
-    <t>21.3.2016</t>
-  </si>
-  <si>
     <t>VERN-R-A</t>
   </si>
   <si>
-    <t>27.1.2016</t>
-  </si>
-  <si>
     <t>HIMR-R-A;HMST;HUPZ;LEDO-R-A;LRH;PLAG;TUHO</t>
   </si>
   <si>
     <t>LKRI;MAIS;OPTE;PTKM;RIZO;TPNG;VERN</t>
   </si>
   <si>
-    <t>21.9.2015</t>
-  </si>
-  <si>
-    <t>11.8.2015</t>
-  </si>
-  <si>
     <t>(PODR uvrštava nove dionice)</t>
   </si>
   <si>
@@ -309,63 +267,33 @@
     <t>TUHO-R-A;LKPC-R-A;HUPZ-R-A;PLAG-R-A;LRH-R-A;HIMR-R-A;HMST-R-A;INGR-R-A</t>
   </si>
   <si>
-    <t>23.3.2015</t>
-  </si>
-  <si>
     <t>RIVP-R-A</t>
   </si>
   <si>
-    <t>27.1.2015</t>
-  </si>
-  <si>
     <t>INGR;HUPZ;LKPC;VIRO</t>
   </si>
   <si>
-    <t>22.9.2014</t>
-  </si>
-  <si>
     <t>VIRO-R-A;HUPZ-R-A;LKPC-R-A;ARNT-R-A;VDKT-R-A</t>
   </si>
   <si>
-    <t>24.3.2014</t>
-  </si>
-  <si>
     <t>DIOK-R-A</t>
   </si>
   <si>
-    <t>27.11.2014</t>
-  </si>
-  <si>
     <t>LKPC;TISK;VDKT;VIRO</t>
   </si>
   <si>
     <t>THNK;ULPL</t>
   </si>
   <si>
-    <t>23.9.2013</t>
-  </si>
-  <si>
-    <t>15.5.2013</t>
-  </si>
-  <si>
-    <t>18.3.2013</t>
-  </si>
-  <si>
     <t>(KNZM-R-A je i dalje ticker)</t>
   </si>
   <si>
     <t>IGH;ULPL</t>
   </si>
   <si>
-    <t>24.9.2012</t>
-  </si>
-  <si>
     <t>LEDO;VPIK;TISK</t>
   </si>
   <si>
-    <t>19.3.2012</t>
-  </si>
-  <si>
     <t>PBZ;LEDO;CKML;INA</t>
   </si>
   <si>
@@ -378,21 +306,12 @@
     <t>ADPL;BLJE;PBZ</t>
   </si>
   <si>
-    <t>21.3.2011</t>
-  </si>
-  <si>
     <t>BLSC-R-A;PBZ;VDKT</t>
   </si>
   <si>
     <t xml:space="preserve">CKML;ISTT-R-A;KNZM-R-A </t>
   </si>
   <si>
-    <t>20.9.2010</t>
-  </si>
-  <si>
-    <t>5.7.2010</t>
-  </si>
-  <si>
     <t>Smanjenje težine dionica društva Belišće d.d.</t>
   </si>
   <si>
@@ -402,9 +321,6 @@
     <t>Broj dionica ZABA povećao se 5 puta</t>
   </si>
   <si>
-    <t>16.9.2011</t>
-  </si>
-  <si>
     <t>povećanje težine dionica Dalekovod d.d. i Luka Ploče d.d</t>
   </si>
   <si>
@@ -430,9 +346,6 @@
   </si>
   <si>
     <t>(Nisu zadovoljili uvjet broja dana trgovanja.)</t>
-  </si>
-  <si>
-    <t>13.1.2012</t>
   </si>
   <si>
     <t>(nisu zadovoljili uvjet broja dana trgovanja)</t>
@@ -534,6 +447,93 @@
   </si>
   <si>
     <t>KOEI-R-A;THNK-R-A;</t>
+  </si>
+  <si>
+    <t>18.3.2019.</t>
+  </si>
+  <si>
+    <t>22.10.2018.</t>
+  </si>
+  <si>
+    <t>24.9.2018.</t>
+  </si>
+  <si>
+    <t>19.3.2018.</t>
+  </si>
+  <si>
+    <t>18.9.2017.</t>
+  </si>
+  <si>
+    <t>19.6.2017.</t>
+  </si>
+  <si>
+    <t>22.5.2017.</t>
+  </si>
+  <si>
+    <t>20.3.2017.</t>
+  </si>
+  <si>
+    <t>21.11.2016.</t>
+  </si>
+  <si>
+    <t>19.9.2016.</t>
+  </si>
+  <si>
+    <t>21.3.2016.</t>
+  </si>
+  <si>
+    <t>27.1.2016.</t>
+  </si>
+  <si>
+    <t>21.9.2015.</t>
+  </si>
+  <si>
+    <t>11.8.2015.</t>
+  </si>
+  <si>
+    <t>23.3.2015.</t>
+  </si>
+  <si>
+    <t>27.1.2015.</t>
+  </si>
+  <si>
+    <t>22.9.2014.</t>
+  </si>
+  <si>
+    <t>24.3.2014.</t>
+  </si>
+  <si>
+    <t>27.11.2014.</t>
+  </si>
+  <si>
+    <t>23.9.2013.</t>
+  </si>
+  <si>
+    <t>15.5.2013.</t>
+  </si>
+  <si>
+    <t>18.3.2013.</t>
+  </si>
+  <si>
+    <t>24.9.2012.</t>
+  </si>
+  <si>
+    <t>19.3.2012.</t>
+  </si>
+  <si>
+    <t>13.1.2012.</t>
+  </si>
+  <si>
+    <t>16.9.2011.</t>
+  </si>
+  <si>
+    <t>21.3.2011.</t>
+  </si>
+  <si>
+    <t>20.9.2010.</t>
+  </si>
+  <si>
+    <t>5.7.2010.</t>
   </si>
 </sst>
 </file>
@@ -842,9 +842,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="2" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -897,6 +894,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normalno" xfId="0" builtinId="0"/>
@@ -1164,7 +1164,7 @@
   <dimension ref="A1:F1000"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="20" style="33" customWidth="1"/>
+    <col min="1" max="1" width="20" style="32" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
     <col min="3" max="3" width="38.140625" customWidth="1"/>
     <col min="4" max="4" width="41.28515625" customWidth="1"/>
@@ -1174,7 +1174,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="27" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -1194,7 +1194,7 @@
       </c>
     </row>
     <row r="2" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="29">
+      <c r="A2" s="28">
         <v>45912</v>
       </c>
       <c r="B2" s="3" t="s">
@@ -1212,7 +1212,7 @@
       <c r="F2" s="6"/>
     </row>
     <row r="3" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="29">
+      <c r="A3" s="28">
         <v>45820</v>
       </c>
       <c r="B3" s="4" t="s">
@@ -1224,7 +1224,7 @@
       </c>
     </row>
     <row r="4" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="29">
+      <c r="A4" s="28">
         <v>45762</v>
       </c>
       <c r="B4" s="3" t="s">
@@ -1237,11 +1237,11 @@
         <v>13</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>152</v>
+        <v>123</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="29">
+      <c r="A5" s="28">
         <v>45728</v>
       </c>
       <c r="B5" s="4" t="s">
@@ -1259,7 +1259,7 @@
       <c r="F5" s="6"/>
     </row>
     <row r="6" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="29">
+      <c r="A6" s="28">
         <v>45639</v>
       </c>
       <c r="B6" s="3" t="s">
@@ -1272,11 +1272,11 @@
         <v>17</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>151</v>
+        <v>122</v>
       </c>
     </row>
     <row r="7" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="29">
+      <c r="A7" s="28">
         <v>45546</v>
       </c>
       <c r="B7" s="4" t="s">
@@ -1294,7 +1294,7 @@
       <c r="F7" s="6"/>
     </row>
     <row r="8" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="29">
+      <c r="A8" s="28">
         <v>45358</v>
       </c>
       <c r="B8" s="3" t="s">
@@ -1312,7 +1312,7 @@
       <c r="F8" s="6"/>
     </row>
     <row r="9" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="29">
+      <c r="A9" s="28">
         <v>45239</v>
       </c>
       <c r="B9" s="4" t="s">
@@ -1326,14 +1326,14 @@
       </c>
     </row>
     <row r="10" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="29">
+      <c r="A10" s="28">
         <v>45175</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C10" s="26" t="s">
-        <v>150</v>
+      <c r="C10" s="25" t="s">
+        <v>121</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>26</v>
@@ -1344,7 +1344,7 @@
       <c r="F10" s="6"/>
     </row>
     <row r="11" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="29">
+      <c r="A11" s="28">
         <v>44992</v>
       </c>
       <c r="B11" s="4" t="s">
@@ -1353,8 +1353,8 @@
       <c r="C11" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D11" s="25" t="s">
-        <v>150</v>
+      <c r="D11" s="24" t="s">
+        <v>121</v>
       </c>
       <c r="E11" s="4" t="s">
         <v>29</v>
@@ -1362,7 +1362,7 @@
       <c r="F11" s="6"/>
     </row>
     <row r="12" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="29">
+      <c r="A12" s="28">
         <v>44902</v>
       </c>
       <c r="B12" s="3" t="s">
@@ -1375,11 +1375,11 @@
         <v>31</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>149</v>
+        <v>120</v>
       </c>
     </row>
     <row r="13" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="29">
+      <c r="A13" s="28">
         <v>44812</v>
       </c>
       <c r="B13" s="4" t="s">
@@ -1397,7 +1397,7 @@
       <c r="F13" s="6"/>
     </row>
     <row r="14" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="29">
+      <c r="A14" s="28">
         <v>44754</v>
       </c>
       <c r="B14" s="3" t="s">
@@ -1410,11 +1410,11 @@
         <v>36</v>
       </c>
       <c r="F14" s="6" t="s">
-        <v>148</v>
+        <v>119</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="29">
+      <c r="A15" s="28">
         <v>44704</v>
       </c>
       <c r="B15" s="4" t="s">
@@ -1428,7 +1428,7 @@
       </c>
     </row>
     <row r="16" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="29">
+      <c r="A16" s="28">
         <v>44659</v>
       </c>
       <c r="B16" s="3" t="s">
@@ -1441,11 +1441,11 @@
         <v>40</v>
       </c>
       <c r="F16" s="6" t="s">
-        <v>147</v>
+        <v>118</v>
       </c>
     </row>
     <row r="17" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="29">
+      <c r="A17" s="28">
         <v>44629</v>
       </c>
       <c r="B17" s="4" t="s">
@@ -1463,7 +1463,7 @@
       <c r="F17" s="6"/>
     </row>
     <row r="18" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="29">
+      <c r="A18" s="28">
         <v>44621</v>
       </c>
       <c r="B18" s="3" t="s">
@@ -1476,11 +1476,11 @@
         <v>45</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>146</v>
+        <v>117</v>
       </c>
     </row>
     <row r="19" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="29">
+      <c r="A19" s="28">
         <v>44448</v>
       </c>
       <c r="B19" s="4" t="s">
@@ -1498,7 +1498,7 @@
       <c r="F19" s="6"/>
     </row>
     <row r="20" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="29">
+      <c r="A20" s="28">
         <v>44264</v>
       </c>
       <c r="B20" s="3" t="s">
@@ -1516,7 +1516,7 @@
       <c r="F20" s="6"/>
     </row>
     <row r="21" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="29">
+      <c r="A21" s="28">
         <v>44082</v>
       </c>
       <c r="B21" s="4" t="s">
@@ -1534,7 +1534,7 @@
       <c r="F21" s="6"/>
     </row>
     <row r="22" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="29">
+      <c r="A22" s="28">
         <v>43901</v>
       </c>
       <c r="B22" s="3" t="s">
@@ -1552,7 +1552,7 @@
       <c r="F22" s="6"/>
     </row>
     <row r="23" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="29">
+      <c r="A23" s="28">
         <v>43718</v>
       </c>
       <c r="B23" s="4" t="s">
@@ -1567,7 +1567,7 @@
       <c r="F23" s="6"/>
     </row>
     <row r="24" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="29">
+      <c r="A24" s="28">
         <v>43535</v>
       </c>
       <c r="B24" s="3" t="s">
@@ -1578,30 +1578,30 @@
       </c>
       <c r="D24" s="3"/>
       <c r="E24" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="F24" s="6"/>
+    </row>
+    <row r="25" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="28">
+        <v>43532</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C25" s="4" t="s">
         <v>60</v>
-      </c>
-      <c r="F24" s="6"/>
-    </row>
-    <row r="25" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="29">
-        <v>43532</v>
-      </c>
-      <c r="B25" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C25" s="4" t="s">
-        <v>61</v>
       </c>
       <c r="D25" s="4" t="s">
         <v>59</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>60</v>
+        <v>126</v>
       </c>
       <c r="F25" s="6"/>
     </row>
     <row r="26" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="29">
+      <c r="A26" s="28">
         <v>43385</v>
       </c>
       <c r="B26" s="3" t="s">
@@ -1610,194 +1610,194 @@
       <c r="C26" s="3"/>
       <c r="D26" s="3"/>
       <c r="E26" s="7" t="s">
-        <v>62</v>
+        <v>127</v>
       </c>
       <c r="F26" s="6" t="s">
-        <v>145</v>
+        <v>116</v>
       </c>
     </row>
     <row r="27" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="29">
+      <c r="A27" s="28">
         <v>43349</v>
       </c>
       <c r="B27" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D27" s="4" t="s">
         <v>57</v>
       </c>
       <c r="E27" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="F27" s="6"/>
+    </row>
+    <row r="28" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="28">
+        <v>43166</v>
+      </c>
+      <c r="B28" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="E28" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="F28" s="6"/>
+    </row>
+    <row r="29" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="28">
+        <v>42986</v>
+      </c>
+      <c r="B29" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="C29" s="4" t="s">
         <v>64</v>
       </c>
-      <c r="F27" s="6"/>
-    </row>
-    <row r="28" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="29">
-        <v>43166</v>
-      </c>
-      <c r="B28" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="C28" s="3" t="s">
+      <c r="D29" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="D28" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="E28" s="7" t="s">
-        <v>67</v>
-      </c>
-      <c r="F28" s="6"/>
-    </row>
-    <row r="29" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="29">
-        <v>42986</v>
-      </c>
-      <c r="B29" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="C29" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="D29" s="4" t="s">
-        <v>69</v>
-      </c>
       <c r="E29" s="5" t="s">
-        <v>70</v>
+        <v>130</v>
       </c>
       <c r="F29" s="6"/>
     </row>
     <row r="30" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="29">
+      <c r="A30" s="28">
         <v>42895</v>
       </c>
       <c r="B30" s="3" t="s">
         <v>11</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="D30" s="3"/>
       <c r="E30" s="7" t="s">
-        <v>72</v>
+        <v>131</v>
       </c>
       <c r="F30" s="6" t="s">
-        <v>143</v>
+        <v>114</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="29">
+      <c r="A31" s="28">
         <v>42863</v>
       </c>
       <c r="B31" s="4" t="s">
         <v>11</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="D31" s="4"/>
       <c r="E31" s="5" t="s">
-        <v>74</v>
+        <v>132</v>
       </c>
       <c r="F31" s="6" t="s">
-        <v>142</v>
+        <v>113</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="30">
+      <c r="A32" s="29">
         <v>42800</v>
       </c>
       <c r="B32" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="D32" s="21" t="s">
-        <v>132</v>
+        <v>68</v>
+      </c>
+      <c r="D32" s="20" t="s">
+        <v>104</v>
       </c>
       <c r="E32" s="7" t="s">
-        <v>76</v>
+        <v>133</v>
       </c>
       <c r="F32" s="6"/>
     </row>
     <row r="33" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="30">
+      <c r="A33" s="29">
         <v>42682</v>
       </c>
       <c r="B33" s="4" t="s">
         <v>11</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="D33" s="4"/>
       <c r="E33" s="5" t="s">
-        <v>78</v>
+        <v>134</v>
       </c>
       <c r="F33" s="6" t="s">
-        <v>141</v>
+        <v>112</v>
       </c>
     </row>
     <row r="34" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="30">
+      <c r="A34" s="29">
         <v>42621</v>
       </c>
       <c r="B34" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>79</v>
-      </c>
-      <c r="D34" s="20" t="s">
-        <v>80</v>
+        <v>70</v>
+      </c>
+      <c r="D34" s="19" t="s">
+        <v>71</v>
       </c>
       <c r="E34" s="7" t="s">
-        <v>81</v>
+        <v>135</v>
       </c>
       <c r="F34" s="6"/>
     </row>
     <row r="35" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="30">
+      <c r="A35" s="29">
         <v>42432</v>
       </c>
       <c r="B35" s="4" t="s">
         <v>6</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="D35" s="20" t="s">
-        <v>83</v>
+        <v>72</v>
+      </c>
+      <c r="D35" s="19" t="s">
+        <v>73</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>84</v>
+        <v>136</v>
       </c>
       <c r="F35" s="6"/>
     </row>
     <row r="36" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="30">
+      <c r="A36" s="29">
         <v>42389</v>
       </c>
       <c r="B36" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C36" s="24" t="s">
-        <v>85</v>
+      <c r="C36" s="23" t="s">
+        <v>74</v>
       </c>
       <c r="D36" s="3"/>
       <c r="E36" s="7" t="s">
-        <v>86</v>
+        <v>137</v>
       </c>
       <c r="F36" s="6" t="s">
-        <v>140</v>
+        <v>111</v>
       </c>
     </row>
     <row r="37" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="29">
+      <c r="A37" s="28">
         <v>42304</v>
       </c>
       <c r="B37" s="12" t="s">
@@ -1806,32 +1806,32 @@
       <c r="C37" s="9"/>
       <c r="D37" s="12"/>
       <c r="E37" s="13" t="s">
-        <v>123</v>
+        <v>96</v>
       </c>
       <c r="F37" s="6" t="s">
-        <v>139</v>
+        <v>110</v>
       </c>
     </row>
     <row r="38" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="30">
+      <c r="A38" s="29">
         <v>42251</v>
       </c>
       <c r="B38" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C38" s="20" t="s">
-        <v>87</v>
-      </c>
-      <c r="D38" s="25" t="s">
-        <v>88</v>
+      <c r="C38" s="19" t="s">
+        <v>75</v>
+      </c>
+      <c r="D38" s="24" t="s">
+        <v>76</v>
       </c>
       <c r="E38" s="5" t="s">
-        <v>89</v>
+        <v>138</v>
       </c>
       <c r="F38" s="6"/>
     </row>
     <row r="39" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="30">
+      <c r="A39" s="29">
         <v>42216</v>
       </c>
       <c r="B39" s="3" t="s">
@@ -1840,124 +1840,124 @@
       <c r="C39" s="3"/>
       <c r="D39" s="3"/>
       <c r="E39" s="7" t="s">
-        <v>90</v>
+        <v>139</v>
       </c>
       <c r="F39" s="6" t="s">
-        <v>91</v>
+        <v>77</v>
       </c>
     </row>
     <row r="40" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="30">
+      <c r="A40" s="29">
         <v>42069</v>
       </c>
-      <c r="B40" s="25" t="s">
+      <c r="B40" s="24" t="s">
         <v>6</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>93</v>
+        <v>79</v>
       </c>
       <c r="E40" s="5" t="s">
-        <v>94</v>
+        <v>140</v>
       </c>
       <c r="F40" s="6" t="s">
-        <v>138</v>
+        <v>109</v>
       </c>
     </row>
     <row r="41" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="30">
+      <c r="A41" s="29">
         <v>42023</v>
       </c>
       <c r="B41" s="3" t="s">
         <v>11</v>
       </c>
       <c r="C41" s="3"/>
-      <c r="D41" s="17" t="s">
-        <v>95</v>
+      <c r="D41" s="16" t="s">
+        <v>80</v>
       </c>
       <c r="E41" s="7" t="s">
-        <v>96</v>
+        <v>141</v>
       </c>
       <c r="F41" s="6" t="s">
-        <v>137</v>
+        <v>108</v>
       </c>
     </row>
     <row r="42" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="30">
+      <c r="A42" s="29">
         <v>41892</v>
       </c>
       <c r="B42" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C42" s="17" t="s">
-        <v>97</v>
-      </c>
-      <c r="D42" s="17" t="s">
-        <v>131</v>
+      <c r="C42" s="16" t="s">
+        <v>81</v>
+      </c>
+      <c r="D42" s="16" t="s">
+        <v>103</v>
       </c>
       <c r="E42" s="5" t="s">
-        <v>98</v>
+        <v>142</v>
       </c>
       <c r="F42" s="6"/>
     </row>
     <row r="43" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="30">
+      <c r="A43" s="29">
         <v>41705</v>
       </c>
       <c r="B43" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C43" s="26" t="s">
-        <v>154</v>
+      <c r="C43" s="25" t="s">
+        <v>125</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>99</v>
+        <v>82</v>
       </c>
       <c r="E43" s="7" t="s">
-        <v>100</v>
+        <v>143</v>
       </c>
       <c r="F43" s="6"/>
     </row>
     <row r="44" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="30">
+      <c r="A44" s="29">
         <v>41605</v>
       </c>
       <c r="B44" s="4" t="s">
         <v>11</v>
       </c>
       <c r="C44" s="4" t="s">
-        <v>101</v>
+        <v>83</v>
       </c>
       <c r="D44" s="4"/>
       <c r="E44" s="5" t="s">
-        <v>102</v>
+        <v>144</v>
       </c>
       <c r="F44" s="6" t="s">
-        <v>144</v>
+        <v>115</v>
       </c>
     </row>
     <row r="45" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="30">
+      <c r="A45" s="29">
         <v>41523</v>
       </c>
       <c r="B45" s="3" t="s">
         <v>6</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>103</v>
+        <v>84</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>104</v>
+        <v>85</v>
       </c>
       <c r="E45" s="7" t="s">
-        <v>105</v>
+        <v>145</v>
       </c>
       <c r="F45" s="6"/>
     </row>
     <row r="46" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="30">
+      <c r="A46" s="29">
         <v>41401</v>
       </c>
       <c r="B46" s="4" t="s">
@@ -1966,160 +1966,160 @@
       <c r="C46" s="4"/>
       <c r="D46" s="4"/>
       <c r="E46" s="5" t="s">
-        <v>106</v>
+        <v>146</v>
       </c>
       <c r="F46" s="14" t="s">
-        <v>130</v>
+        <v>102</v>
       </c>
     </row>
     <row r="47" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="30">
+      <c r="A47" s="29">
         <v>41339</v>
       </c>
       <c r="B47" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="C47" s="16" t="s">
-        <v>128</v>
-      </c>
-      <c r="D47" s="16" t="s">
-        <v>129</v>
+      <c r="C47" s="15" t="s">
+        <v>100</v>
+      </c>
+      <c r="D47" s="15" t="s">
+        <v>101</v>
       </c>
       <c r="E47" s="7" t="s">
+        <v>147</v>
+      </c>
+      <c r="F47" s="8" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="29">
+        <v>41157</v>
+      </c>
+      <c r="B48" s="17" t="s">
+        <v>6</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="D48" s="16" t="s">
+        <v>99</v>
+      </c>
+      <c r="E48" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="F48" s="6"/>
+    </row>
+    <row r="49" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="29">
+        <v>40974</v>
+      </c>
+      <c r="B49" s="18" t="s">
+        <v>6</v>
+      </c>
+      <c r="C49" s="25" t="s">
+        <v>124</v>
+      </c>
+      <c r="D49" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="E49" s="7" t="s">
+        <v>149</v>
+      </c>
+      <c r="F49" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="F47" s="8" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="30">
-        <v>41157</v>
-      </c>
-      <c r="B48" s="18" t="s">
-        <v>6</v>
-      </c>
-      <c r="C48" s="4" t="s">
-        <v>109</v>
-      </c>
-      <c r="D48" s="17" t="s">
-        <v>127</v>
-      </c>
-      <c r="E48" s="5" t="s">
-        <v>110</v>
-      </c>
-      <c r="F48" s="6"/>
-    </row>
-    <row r="49" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="30">
-        <v>40974</v>
-      </c>
-      <c r="B49" s="19" t="s">
-        <v>6</v>
-      </c>
-      <c r="C49" s="26" t="s">
-        <v>153</v>
-      </c>
-      <c r="D49" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="E49" s="7" t="s">
-        <v>112</v>
-      </c>
-      <c r="F49" s="8" t="s">
-        <v>136</v>
-      </c>
     </row>
     <row r="50" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="31">
+      <c r="A50" s="30">
         <v>40912</v>
       </c>
-      <c r="B50" s="18" t="s">
+      <c r="B50" s="17" t="s">
         <v>11</v>
       </c>
       <c r="C50" s="4"/>
       <c r="D50" s="4"/>
-      <c r="E50" s="23" t="s">
-        <v>135</v>
+      <c r="E50" s="22" t="s">
+        <v>150</v>
       </c>
       <c r="F50" s="14" t="s">
-        <v>126</v>
+        <v>98</v>
       </c>
     </row>
     <row r="51" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="31">
+      <c r="A51" s="30">
         <v>40792</v>
       </c>
-      <c r="B51" s="19" t="s">
-        <v>6</v>
-      </c>
-      <c r="C51" s="16" t="s">
-        <v>113</v>
+      <c r="B51" s="18" t="s">
+        <v>6</v>
+      </c>
+      <c r="C51" s="15" t="s">
+        <v>89</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="E51" s="15" t="s">
-        <v>125</v>
+        <v>90</v>
+      </c>
+      <c r="E51" s="33" t="s">
+        <v>151</v>
       </c>
       <c r="F51" s="8" t="s">
-        <v>134</v>
+        <v>106</v>
       </c>
     </row>
     <row r="52" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="31">
+      <c r="A52" s="30">
         <v>40750</v>
       </c>
-      <c r="B52" s="18" t="s">
+      <c r="B52" s="17" t="s">
         <v>11</v>
       </c>
       <c r="C52" s="4"/>
       <c r="D52" s="4"/>
       <c r="E52" s="5"/>
       <c r="F52" s="14" t="s">
-        <v>124</v>
+        <v>97</v>
       </c>
     </row>
     <row r="53" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="31">
+      <c r="A53" s="30">
         <v>40606</v>
       </c>
-      <c r="B53" s="19" t="s">
+      <c r="B53" s="18" t="s">
         <v>6</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>115</v>
+        <v>91</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>116</v>
+        <v>92</v>
       </c>
       <c r="E53" s="7" t="s">
-        <v>117</v>
-      </c>
-      <c r="F53" s="22" t="s">
-        <v>133</v>
+        <v>152</v>
+      </c>
+      <c r="F53" s="21" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="54" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="31">
+      <c r="A54" s="30">
         <v>40429</v>
       </c>
-      <c r="B54" s="18" t="s">
+      <c r="B54" s="17" t="s">
         <v>6</v>
       </c>
       <c r="C54" s="4" t="s">
-        <v>118</v>
+        <v>93</v>
       </c>
       <c r="D54" s="4" t="s">
-        <v>119</v>
+        <v>94</v>
       </c>
       <c r="E54" s="5" t="s">
-        <v>120</v>
+        <v>153</v>
       </c>
       <c r="F54" s="6"/>
     </row>
     <row r="55" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="32">
+      <c r="A55" s="31">
         <v>40339</v>
       </c>
       <c r="B55" s="10" t="s">
@@ -2128,10 +2128,10 @@
       <c r="C55" s="10"/>
       <c r="D55" s="10"/>
       <c r="E55" s="11" t="s">
-        <v>121</v>
-      </c>
-      <c r="F55" s="27" t="s">
-        <v>122</v>
+        <v>154</v>
+      </c>
+      <c r="F55" s="26" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="56" spans="1:6" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>

</xml_diff>